<commit_message>
Mise à jour fiches et TO GPME
</commit_message>
<xml_diff>
--- a/bts-gpme/tp-1083/ressources/R02_Registre_evenements_SST_et_cotation.xlsx
+++ b/bts-gpme/tp-1083/ressources/R02_Registre_evenements_SST_et_cotation.xlsx
@@ -2,8 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Incidents" sheetId="1" r:id="R2dbb4cf445bc4b12"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Grille_DUERP" sheetId="2" r:id="R18cb67ef642c4c5e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Incidents" sheetId="1" r:id="Reb2acf3e94ab4fad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Grille_DUERP" sheetId="2" r:id="R0b1738b0cbeb4f6c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Contrôle_données" sheetId="3" r:id="R3dc0c143f630465c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -17,7 +18,7 @@
   <x:numFmts count="1">
     <x:numFmt numFmtId="200" formatCode="dd/mm/yyyy"/>
   </x:numFmts>
-  <x:fonts count="5">
+  <x:fonts count="6">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -45,8 +46,14 @@
       <x:sz val="11"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF7F6000"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="6">
+  <x:fills count="8">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -73,6 +80,16 @@
         <x:fgColor rgb="FFFFF2CC"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF2F5F78"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="2">
     <x:border/>
@@ -81,7 +98,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="25">
+  <x:cellXfs count="35">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -134,6 +151,28 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -889,9 +928,7 @@
       <x:c r="I18" s="16" t="str">
         <x:v>Arrêt d'urgence machine</x:v>
       </x:c>
-      <x:c r="J18" s="16" t="str">
-        <x:v>Ligne potentiellement dupliquée dans le registre.</x:v>
-      </x:c>
+      <x:c r="J18" s="16" t="str"/>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="16" t="str">
@@ -931,7 +968,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R13d50b1d3b0941a2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R03d4905a5261439a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1052,7 +1089,7 @@
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="14" t="str">
-        <x:v>Score brut P×G</x:v>
+        <x:v>Criticité P×G</x:v>
       </x:c>
       <x:c r="B10" s="14" t="str">
         <x:v>1 à 5</x:v>
@@ -1104,17 +1141,17 @@
       <x:c r="C14" s="16"/>
       <x:c r="D14" s="16"/>
     </x:row>
-    <x:row r="15">
+    <x:row r="15" ht="62" customHeight="1">
       <x:c r="A15" s="16" t="str">
         <x:v>Consigne</x:v>
       </x:c>
       <x:c r="B15" s="16" t="str">
-        <x:v>Tenez compte des mesures existantes pour réévaluer le risque et proposer les actions complémentaires.</x:v>
+        <x:v>Tenez compte des mesures existantes pour réévaluer le risque et proposer les actions complémentaires. Une mesure existante n’est pas nécessairement efficace.</x:v>
       </x:c>
       <x:c r="C15" s="16"/>
       <x:c r="D15" s="16"/>
     </x:row>
-    <x:row r="16">
+    <x:row r="16" ht="42" customHeight="1">
       <x:c r="A16" s="24" t="str">
         <x:v>Règle de vigilance</x:v>
       </x:c>
@@ -1124,7 +1161,7 @@
       <x:c r="C16" s="24"/>
       <x:c r="D16" s="24"/>
     </x:row>
-    <x:row r="17">
+    <x:row r="17" ht="42" customHeight="1">
       <x:c r="A17" s="16" t="str">
         <x:v>Contrôle</x:v>
       </x:c>
@@ -1133,6 +1170,14 @@
       </x:c>
       <x:c r="C17" s="16"/>
       <x:c r="D17" s="16"/>
+    </x:row>
+    <x:row r="18" ht="62" customHeight="1">
+      <x:c r="A18" t="str">
+        <x:v>Consigne</x:v>
+      </x:c>
+      <x:c r="B18" s="16" t="str">
+        <x:v>La gravité s’apprécie à partir du dommage potentiel plausible, et non seulement du dommage effectivement observé lors du dernier événement.</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1140,4 +1185,159 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="16" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="30" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="24" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="36" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="34" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="34" customHeight="1">
+      <x:c r="A1" s="28" t="str">
+        <x:v>TRACE DE CONTRÔLE — consignez les anomalies repérées avant tout calcul ; ne supprimez aucune donnée sans justification.</x:v>
+      </x:c>
+      <x:c r="B1" s="28"/>
+      <x:c r="C1" s="28"/>
+      <x:c r="D1" s="28"/>
+      <x:c r="E1" s="28"/>
+    </x:row>
+    <x:row r="3" ht="28" customHeight="1">
+      <x:c r="A3" s="33" t="str">
+        <x:v>ID concerné</x:v>
+      </x:c>
+      <x:c r="B3" s="33" t="str">
+        <x:v>Anomalie constatée</x:v>
+      </x:c>
+      <x:c r="C3" s="33" t="str">
+        <x:v>Décision prise</x:v>
+      </x:c>
+      <x:c r="D3" s="33" t="str">
+        <x:v>Justification</x:v>
+      </x:c>
+      <x:c r="E3" s="33" t="str">
+        <x:v>Information à confirmer</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="38" customHeight="1">
+      <x:c r="A4" s="34" t="str"/>
+      <x:c r="B4" s="34" t="str"/>
+      <x:c r="C4" s="34" t="str"/>
+      <x:c r="D4" s="34" t="str"/>
+      <x:c r="E4" s="34" t="str"/>
+    </x:row>
+    <x:row r="5" ht="38" customHeight="1">
+      <x:c r="A5" s="34" t="str"/>
+      <x:c r="B5" s="34" t="str"/>
+      <x:c r="C5" s="34" t="str"/>
+      <x:c r="D5" s="34" t="str"/>
+      <x:c r="E5" s="34" t="str"/>
+    </x:row>
+    <x:row r="6" ht="38" customHeight="1">
+      <x:c r="A6" s="34" t="str"/>
+      <x:c r="B6" s="34" t="str"/>
+      <x:c r="C6" s="34" t="str"/>
+      <x:c r="D6" s="34" t="str"/>
+      <x:c r="E6" s="34" t="str"/>
+    </x:row>
+    <x:row r="7" ht="38" customHeight="1">
+      <x:c r="A7" s="34" t="str"/>
+      <x:c r="B7" s="34" t="str"/>
+      <x:c r="C7" s="34" t="str"/>
+      <x:c r="D7" s="34" t="str"/>
+      <x:c r="E7" s="34" t="str"/>
+    </x:row>
+    <x:row r="8" ht="38" customHeight="1">
+      <x:c r="A8" s="34" t="str"/>
+      <x:c r="B8" s="34" t="str"/>
+      <x:c r="C8" s="34" t="str"/>
+      <x:c r="D8" s="34" t="str"/>
+      <x:c r="E8" s="34" t="str"/>
+    </x:row>
+    <x:row r="9" ht="38" customHeight="1">
+      <x:c r="A9" s="34" t="str"/>
+      <x:c r="B9" s="34" t="str"/>
+      <x:c r="C9" s="34" t="str"/>
+      <x:c r="D9" s="34" t="str"/>
+      <x:c r="E9" s="34" t="str"/>
+    </x:row>
+    <x:row r="10" ht="38" customHeight="1">
+      <x:c r="A10" s="34" t="str"/>
+      <x:c r="B10" s="34" t="str"/>
+      <x:c r="C10" s="34" t="str"/>
+      <x:c r="D10" s="34" t="str"/>
+      <x:c r="E10" s="34" t="str"/>
+    </x:row>
+    <x:row r="11" ht="38" customHeight="1">
+      <x:c r="A11" s="34" t="str"/>
+      <x:c r="B11" s="34" t="str"/>
+      <x:c r="C11" s="34" t="str"/>
+      <x:c r="D11" s="34" t="str"/>
+      <x:c r="E11" s="34" t="str"/>
+    </x:row>
+    <x:row r="12" ht="38" customHeight="1">
+      <x:c r="A12" s="34" t="str"/>
+      <x:c r="B12" s="34" t="str"/>
+      <x:c r="C12" s="34" t="str"/>
+      <x:c r="D12" s="34" t="str"/>
+      <x:c r="E12" s="34" t="str"/>
+    </x:row>
+    <x:row r="13" ht="38" customHeight="1">
+      <x:c r="A13" s="34" t="str"/>
+      <x:c r="B13" s="34" t="str"/>
+      <x:c r="C13" s="34" t="str"/>
+      <x:c r="D13" s="34" t="str"/>
+      <x:c r="E13" s="34" t="str"/>
+    </x:row>
+    <x:row r="14" ht="38" customHeight="1">
+      <x:c r="A14" s="34" t="str"/>
+      <x:c r="B14" s="34" t="str"/>
+      <x:c r="C14" s="34" t="str"/>
+      <x:c r="D14" s="34" t="str"/>
+      <x:c r="E14" s="34" t="str"/>
+    </x:row>
+    <x:row r="15" ht="38" customHeight="1">
+      <x:c r="A15" s="34" t="str"/>
+      <x:c r="B15" s="34" t="str"/>
+      <x:c r="C15" s="34" t="str"/>
+      <x:c r="D15" s="34" t="str"/>
+      <x:c r="E15" s="34" t="str"/>
+    </x:row>
+    <x:row r="16" ht="38" customHeight="1">
+      <x:c r="A16" s="34" t="str"/>
+      <x:c r="B16" s="34" t="str"/>
+      <x:c r="C16" s="34" t="str"/>
+      <x:c r="D16" s="34" t="str"/>
+      <x:c r="E16" s="34" t="str"/>
+    </x:row>
+    <x:row r="17" ht="38" customHeight="1">
+      <x:c r="A17" s="34" t="str"/>
+      <x:c r="B17" s="34" t="str"/>
+      <x:c r="C17" s="34" t="str"/>
+      <x:c r="D17" s="34" t="str"/>
+      <x:c r="E17" s="34" t="str"/>
+    </x:row>
+    <x:row r="18" ht="38" customHeight="1">
+      <x:c r="A18" s="34" t="str"/>
+      <x:c r="B18" s="34" t="str"/>
+      <x:c r="C18" s="34" t="str"/>
+      <x:c r="D18" s="34" t="str"/>
+      <x:c r="E18" s="34" t="str"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:E1"/>
+  </x:mergeCells>
+  <x:dataValidations count="1">
+    <x:dataValidation type="list" sqref="C4:C18">
+      <x:formula1>"Conserver,Corriger,Écarter temporairement,À confirmer"</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>